<commit_message>
feat: memecah tambah pagu menjadi penugasan dan inisiatif
</commit_message>
<xml_diff>
--- a/db.xlsx
+++ b/db.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BK\OneDrive - UGM 365\Desktop\verifikasi-online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73ED0B9A-6E50-4229-9410-95A0490C428B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A80717-36DE-4AAC-AA0C-A1BB2EE6EACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{14108520-BF54-4EAA-92D2-D404123A5DCA}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12250" uniqueCount="1477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12250" uniqueCount="1478">
   <si>
     <t>unit_id</t>
   </si>
@@ -4474,6 +4474,9 @@
   </si>
   <si>
     <t>Tambah Pagu - Inisiatif</t>
+  </si>
+  <si>
+    <t>Tambah Pagu - Penugasan</t>
   </si>
 </sst>
 </file>
@@ -7714,7 +7717,7 @@
     <col min="4" max="4" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -25323,8 +25326,8 @@
       <c r="F755" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G755" s="4" t="s">
-        <v>1468</v>
+      <c r="G755" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K755" s="8" t="s">
         <v>1473</v>
@@ -26252,8 +26255,8 @@
       <c r="F793" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G793" s="4" t="s">
-        <v>1468</v>
+      <c r="G793" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K793" s="8" t="s">
         <v>1473</v>
@@ -26460,8 +26463,8 @@
       <c r="F801" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G801" s="4" t="s">
-        <v>1468</v>
+      <c r="G801" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K801" s="8" t="s">
         <v>1473</v>
@@ -27292,8 +27295,8 @@
       <c r="F833" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G833" s="4" t="s">
-        <v>1468</v>
+      <c r="G833" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K833" s="8" t="s">
         <v>1473</v>
@@ -29198,8 +29201,8 @@
       <c r="F907" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G907" s="4" t="s">
-        <v>1468</v>
+      <c r="G907" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K907" s="8" t="s">
         <v>1473</v>
@@ -29224,8 +29227,8 @@
       <c r="F908" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G908" s="4" t="s">
-        <v>1468</v>
+      <c r="G908" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K908" s="8" t="s">
         <v>1473</v>
@@ -29302,8 +29305,8 @@
       <c r="F911" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G911" s="4" t="s">
-        <v>1468</v>
+      <c r="G911" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K911" s="8" t="s">
         <v>1473</v>
@@ -29328,8 +29331,8 @@
       <c r="F912" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G912" s="4" t="s">
-        <v>1468</v>
+      <c r="G912" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K912" s="8" t="s">
         <v>1473</v>
@@ -29432,8 +29435,8 @@
       <c r="F916" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G916" s="4" t="s">
-        <v>1468</v>
+      <c r="G916" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K916" s="8" t="s">
         <v>1473</v>
@@ -29458,8 +29461,8 @@
       <c r="F917" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G917" s="4" t="s">
-        <v>1468</v>
+      <c r="G917" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K917" s="8" t="s">
         <v>1473</v>
@@ -29611,8 +29614,8 @@
       <c r="F923" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G923" s="4" t="s">
-        <v>1468</v>
+      <c r="G923" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K923" s="8" t="s">
         <v>1473</v>
@@ -29787,8 +29790,8 @@
       <c r="F930" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G930" s="4" t="s">
-        <v>1468</v>
+      <c r="G930" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K930" s="8" t="s">
         <v>1473</v>
@@ -29917,8 +29920,8 @@
       <c r="F935" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G935" s="4" t="s">
-        <v>1468</v>
+      <c r="G935" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K935" s="8" t="s">
         <v>1473</v>
@@ -30307,8 +30310,8 @@
       <c r="F950" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G950" s="4" t="s">
-        <v>1468</v>
+      <c r="G950" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K950" s="8" t="s">
         <v>1473</v>
@@ -30333,8 +30336,8 @@
       <c r="F951" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G951" s="4" t="s">
-        <v>1468</v>
+      <c r="G951" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K951" s="8" t="s">
         <v>1473</v>
@@ -30460,8 +30463,8 @@
       <c r="F956" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G956" s="4" t="s">
-        <v>1468</v>
+      <c r="G956" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K956" s="8" t="s">
         <v>1473</v>
@@ -30486,8 +30489,8 @@
       <c r="F957" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G957" s="4" t="s">
-        <v>1468</v>
+      <c r="G957" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K957" s="8" t="s">
         <v>1473</v>
@@ -30512,8 +30515,8 @@
       <c r="F958" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G958" s="4" t="s">
-        <v>1468</v>
+      <c r="G958" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K958" s="8" t="s">
         <v>1473</v>
@@ -30538,8 +30541,8 @@
       <c r="F959" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G959" s="4" t="s">
-        <v>1468</v>
+      <c r="G959" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K959" s="8" t="s">
         <v>1473</v>
@@ -30613,8 +30616,8 @@
       <c r="F962" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G962" s="4" t="s">
-        <v>1468</v>
+      <c r="G962" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K962" s="8" t="s">
         <v>1473</v>
@@ -30639,8 +30642,8 @@
       <c r="F963" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G963" s="4" t="s">
-        <v>1468</v>
+      <c r="G963" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K963" s="8" t="s">
         <v>1473</v>
@@ -30717,8 +30720,8 @@
       <c r="F966" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G966" s="4" t="s">
-        <v>1468</v>
+      <c r="G966" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K966" s="8" t="s">
         <v>1473</v>
@@ -30769,8 +30772,8 @@
       <c r="F968" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G968" s="4" t="s">
-        <v>1468</v>
+      <c r="G968" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K968" s="8" t="s">
         <v>1473</v>
@@ -30821,8 +30824,8 @@
       <c r="F970" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G970" s="4" t="s">
-        <v>1468</v>
+      <c r="G970" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K970" s="8" t="s">
         <v>1473</v>
@@ -30922,8 +30925,8 @@
       <c r="F974" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G974" s="4" t="s">
-        <v>1468</v>
+      <c r="G974" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K974" s="8" t="s">
         <v>1473</v>
@@ -30974,8 +30977,8 @@
       <c r="F976" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G976" s="4" t="s">
-        <v>1468</v>
+      <c r="G976" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K976" s="8" t="s">
         <v>1473</v>
@@ -31000,8 +31003,8 @@
       <c r="F977" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G977" s="4" t="s">
-        <v>1468</v>
+      <c r="G977" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K977" s="8" t="s">
         <v>1473</v>
@@ -32490,8 +32493,8 @@
       <c r="F1035" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1035" s="4" t="s">
-        <v>1468</v>
+      <c r="G1035" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1035" s="8" t="s">
         <v>1473</v>
@@ -32516,8 +32519,8 @@
       <c r="F1036" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1036" s="4" t="s">
-        <v>1468</v>
+      <c r="G1036" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1036" s="8" t="s">
         <v>1473</v>
@@ -32568,8 +32571,8 @@
       <c r="F1038" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1038" s="4" t="s">
-        <v>1468</v>
+      <c r="G1038" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1038" s="8" t="s">
         <v>1473</v>
@@ -32672,8 +32675,8 @@
       <c r="F1042" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1042" s="4" t="s">
-        <v>1468</v>
+      <c r="G1042" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1042" s="8" t="s">
         <v>1473</v>
@@ -32724,8 +32727,8 @@
       <c r="F1044" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1044" s="4" t="s">
-        <v>1468</v>
+      <c r="G1044" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1044" s="8" t="s">
         <v>1473</v>
@@ -33033,8 +33036,8 @@
       <c r="F1056" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1056" s="4" t="s">
-        <v>1468</v>
+      <c r="G1056" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1056" s="8" t="s">
         <v>1473</v>
@@ -33215,8 +33218,8 @@
       <c r="F1063" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1063" s="4" t="s">
-        <v>1468</v>
+      <c r="G1063" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1063" s="8" t="s">
         <v>1473</v>
@@ -33267,8 +33270,8 @@
       <c r="F1065" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1065" s="4" t="s">
-        <v>1468</v>
+      <c r="G1065" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1065" s="8" t="s">
         <v>1473</v>
@@ -33345,8 +33348,8 @@
       <c r="F1068" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1068" s="4" t="s">
-        <v>1468</v>
+      <c r="G1068" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1068" s="8" t="s">
         <v>1473</v>
@@ -33472,8 +33475,8 @@
       <c r="F1073" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1073" s="4" t="s">
-        <v>1468</v>
+      <c r="G1073" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1073" s="8" t="s">
         <v>1473</v>
@@ -33859,8 +33862,8 @@
       <c r="F1088" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1088" s="4" t="s">
-        <v>1468</v>
+      <c r="G1088" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1088" s="8" t="s">
         <v>1473</v>
@@ -33885,8 +33888,8 @@
       <c r="F1089" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1089" s="4" t="s">
-        <v>1468</v>
+      <c r="G1089" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1089" s="8" t="s">
         <v>1473</v>
@@ -33937,8 +33940,8 @@
       <c r="F1091" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1091" s="4" t="s">
-        <v>1468</v>
+      <c r="G1091" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1091" s="8" t="s">
         <v>1473</v>
@@ -34041,8 +34044,8 @@
       <c r="F1095" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1095" s="4" t="s">
-        <v>1468</v>
+      <c r="G1095" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1095" s="8" t="s">
         <v>1473</v>
@@ -34067,8 +34070,8 @@
       <c r="F1096" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1096" s="4" t="s">
-        <v>1468</v>
+      <c r="G1096" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1096" s="8" t="s">
         <v>1473</v>
@@ -34116,8 +34119,8 @@
       <c r="F1098" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1098" s="4" t="s">
-        <v>1468</v>
+      <c r="G1098" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1098" s="8" t="s">
         <v>1473</v>
@@ -34142,8 +34145,8 @@
       <c r="F1099" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1099" s="4" t="s">
-        <v>1468</v>
+      <c r="G1099" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1099" s="8" t="s">
         <v>1473</v>
@@ -34376,8 +34379,8 @@
       <c r="F1108" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1108" s="4" t="s">
-        <v>1468</v>
+      <c r="G1108" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1108" s="8" t="s">
         <v>1473</v>
@@ -34428,8 +34431,8 @@
       <c r="F1110" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1110" s="4" t="s">
-        <v>1468</v>
+      <c r="G1110" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1110" s="8" t="s">
         <v>1473</v>
@@ -34480,8 +34483,8 @@
       <c r="F1112" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1112" s="4" t="s">
-        <v>1468</v>
+      <c r="G1112" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1112" s="8" t="s">
         <v>1473</v>
@@ -34662,8 +34665,8 @@
       <c r="F1119" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1119" s="4" t="s">
-        <v>1468</v>
+      <c r="G1119" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1119" s="8" t="s">
         <v>1473</v>
@@ -34714,8 +34717,8 @@
       <c r="F1121" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1121" s="4" t="s">
-        <v>1468</v>
+      <c r="G1121" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1121" s="8" t="s">
         <v>1473</v>
@@ -34792,8 +34795,8 @@
       <c r="F1124" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1124" s="4" t="s">
-        <v>1468</v>
+      <c r="G1124" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1124" s="8" t="s">
         <v>1473</v>
@@ -34818,8 +34821,8 @@
       <c r="F1125" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1125" s="4" t="s">
-        <v>1468</v>
+      <c r="G1125" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1125" s="8" t="s">
         <v>1473</v>
@@ -35000,8 +35003,8 @@
       <c r="F1132" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1132" s="4" t="s">
-        <v>1468</v>
+      <c r="G1132" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1132" s="8" t="s">
         <v>1473</v>
@@ -36360,8 +36363,8 @@
       <c r="F1185" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1185" s="4" t="s">
-        <v>1468</v>
+      <c r="G1185" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1185" s="8" t="s">
         <v>1473</v>
@@ -36386,8 +36389,8 @@
       <c r="F1186" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1186" s="4" t="s">
-        <v>1468</v>
+      <c r="G1186" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1186" s="8" t="s">
         <v>1473</v>
@@ -36542,8 +36545,8 @@
       <c r="F1192" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1192" s="4" t="s">
-        <v>1468</v>
+      <c r="G1192" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1192" s="8" t="s">
         <v>1473</v>
@@ -36568,8 +36571,8 @@
       <c r="F1193" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1193" s="4" t="s">
-        <v>1468</v>
+      <c r="G1193" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1193" s="8" t="s">
         <v>1473</v>
@@ -36672,8 +36675,8 @@
       <c r="F1197" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1197" s="4" t="s">
-        <v>1468</v>
+      <c r="G1197" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1197" s="8" t="s">
         <v>1473</v>
@@ -36724,8 +36727,8 @@
       <c r="F1199" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1199" s="4" t="s">
-        <v>1468</v>
+      <c r="G1199" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1199" s="8" t="s">
         <v>1473</v>
@@ -36825,8 +36828,8 @@
       <c r="F1203" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1203" s="4" t="s">
-        <v>1468</v>
+      <c r="G1203" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1203" s="8" t="s">
         <v>1473</v>
@@ -36874,8 +36877,8 @@
       <c r="F1205" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1205" s="4" t="s">
-        <v>1468</v>
+      <c r="G1205" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1205" s="8" t="s">
         <v>1473</v>
@@ -37532,8 +37535,8 @@
       <c r="F1231" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1231" s="4" t="s">
-        <v>1468</v>
+      <c r="G1231" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1231" s="8" t="s">
         <v>1473</v>
@@ -37558,8 +37561,8 @@
       <c r="F1232" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1232" s="4" t="s">
-        <v>1468</v>
+      <c r="G1232" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1232" s="8" t="s">
         <v>1473</v>
@@ -37714,8 +37717,8 @@
       <c r="F1238" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1238" s="4" t="s">
-        <v>1468</v>
+      <c r="G1238" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1238" s="8" t="s">
         <v>1473</v>
@@ -37867,8 +37870,8 @@
       <c r="F1244" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1244" s="4" t="s">
-        <v>1468</v>
+      <c r="G1244" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1244" s="8" t="s">
         <v>1473</v>
@@ -37893,8 +37896,8 @@
       <c r="F1245" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1245" s="4" t="s">
-        <v>1468</v>
+      <c r="G1245" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1245" s="8" t="s">
         <v>1473</v>
@@ -37945,8 +37948,8 @@
       <c r="F1247" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1247" s="4" t="s">
-        <v>1468</v>
+      <c r="G1247" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1247" s="8" t="s">
         <v>1473</v>
@@ -37971,8 +37974,8 @@
       <c r="F1248" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1248" s="4" t="s">
-        <v>1468</v>
+      <c r="G1248" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1248" s="8" t="s">
         <v>1473</v>
@@ -37997,8 +38000,8 @@
       <c r="F1249" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1249" s="4" t="s">
-        <v>1468</v>
+      <c r="G1249" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1249" s="8" t="s">
         <v>1473</v>
@@ -38127,8 +38130,8 @@
       <c r="F1254" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1254" s="4" t="s">
-        <v>1468</v>
+      <c r="G1254" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1254" s="8" t="s">
         <v>1473</v>
@@ -38205,8 +38208,8 @@
       <c r="F1257" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1257" s="4" t="s">
-        <v>1468</v>
+      <c r="G1257" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1257" s="8" t="s">
         <v>1473</v>
@@ -38257,8 +38260,8 @@
       <c r="F1259" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1259" s="4" t="s">
-        <v>1468</v>
+      <c r="G1259" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1259" s="8" t="s">
         <v>1473</v>
@@ -38283,8 +38286,8 @@
       <c r="F1260" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1260" s="4" t="s">
-        <v>1468</v>
+      <c r="G1260" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1260" s="8" t="s">
         <v>1473</v>
@@ -38335,8 +38338,8 @@
       <c r="F1262" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1262" s="4" t="s">
-        <v>1468</v>
+      <c r="G1262" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1262" s="8" t="s">
         <v>1473</v>
@@ -38387,8 +38390,8 @@
       <c r="F1264" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1264" s="4" t="s">
-        <v>1468</v>
+      <c r="G1264" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1264" s="8" t="s">
         <v>1473</v>
@@ -38439,8 +38442,8 @@
       <c r="F1266" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1266" s="4" t="s">
-        <v>1468</v>
+      <c r="G1266" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1266" s="8" t="s">
         <v>1473</v>
@@ -38543,8 +38546,8 @@
       <c r="F1270" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1270" s="4" t="s">
-        <v>1468</v>
+      <c r="G1270" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1270" s="8" t="s">
         <v>1473</v>
@@ -38644,8 +38647,8 @@
       <c r="F1274" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1274" s="4" t="s">
-        <v>1468</v>
+      <c r="G1274" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1274" s="8" t="s">
         <v>1473</v>
@@ -38670,8 +38673,8 @@
       <c r="F1275" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1275" s="4" t="s">
-        <v>1468</v>
+      <c r="G1275" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1275" s="8" t="s">
         <v>1473</v>
@@ -39395,8 +39398,8 @@
       <c r="F1303" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1303" s="4" t="s">
-        <v>1468</v>
+      <c r="G1303" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1303" s="8" t="s">
         <v>1473</v>
@@ -39626,8 +39629,8 @@
       <c r="F1312" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1312" s="4" t="s">
-        <v>1468</v>
+      <c r="G1312" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1312" s="8" t="s">
         <v>1473</v>
@@ -39652,8 +39655,8 @@
       <c r="F1313" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1313" s="4" t="s">
-        <v>1468</v>
+      <c r="G1313" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1313" s="8" t="s">
         <v>1473</v>
@@ -39678,8 +39681,8 @@
       <c r="F1314" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1314" s="4" t="s">
-        <v>1468</v>
+      <c r="G1314" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1314" s="8" t="s">
         <v>1473</v>
@@ -39730,8 +39733,8 @@
       <c r="F1316" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1316" s="4" t="s">
-        <v>1468</v>
+      <c r="G1316" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1316" s="8" t="s">
         <v>1473</v>
@@ -40796,8 +40799,8 @@
       <c r="F1357" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1357" s="4" t="s">
-        <v>1468</v>
+      <c r="G1357" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1357" s="8" t="s">
         <v>1473</v>
@@ -40848,8 +40851,8 @@
       <c r="F1359" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1359" s="4" t="s">
-        <v>1468</v>
+      <c r="G1359" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1359" s="8" t="s">
         <v>1473</v>
@@ -40926,8 +40929,8 @@
       <c r="F1362" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1362" s="4" t="s">
-        <v>1468</v>
+      <c r="G1362" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1362" s="8" t="s">
         <v>1473</v>
@@ -41079,8 +41082,8 @@
       <c r="F1368" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1368" s="4" t="s">
-        <v>1468</v>
+      <c r="G1368" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1368" s="8" t="s">
         <v>1473</v>
@@ -41529,8 +41532,8 @@
       <c r="F1386" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1386" s="4" t="s">
-        <v>1468</v>
+      <c r="G1386" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1386" s="8" t="s">
         <v>1473</v>
@@ -41555,8 +41558,8 @@
       <c r="F1387" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1387" s="4" t="s">
-        <v>1468</v>
+      <c r="G1387" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1387" s="8" t="s">
         <v>1473</v>
@@ -43224,8 +43227,8 @@
       <c r="F1452" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1452" s="4" t="s">
-        <v>1468</v>
+      <c r="G1452" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1452" s="8" t="s">
         <v>1473</v>
@@ -43299,8 +43302,8 @@
       <c r="F1455" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1455" s="4" t="s">
-        <v>1468</v>
+      <c r="G1455" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1455" s="8" t="s">
         <v>1473</v>
@@ -43452,8 +43455,8 @@
       <c r="F1461" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1461" s="4" t="s">
-        <v>1468</v>
+      <c r="G1461" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1461" s="8" t="s">
         <v>1473</v>
@@ -43504,8 +43507,8 @@
       <c r="F1463" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1463" s="4" t="s">
-        <v>1468</v>
+      <c r="G1463" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1463" s="8" t="s">
         <v>1473</v>
@@ -43530,8 +43533,8 @@
       <c r="F1464" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1464" s="4" t="s">
-        <v>1468</v>
+      <c r="G1464" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1464" s="8" t="s">
         <v>1473</v>
@@ -43712,8 +43715,8 @@
       <c r="F1471" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1471" s="4" t="s">
-        <v>1468</v>
+      <c r="G1471" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1471" s="8" t="s">
         <v>1473</v>
@@ -43813,8 +43816,8 @@
       <c r="F1475" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1475" s="4" t="s">
-        <v>1468</v>
+      <c r="G1475" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1475" s="8" t="s">
         <v>1473</v>
@@ -43943,8 +43946,8 @@
       <c r="F1480" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1480" s="4" t="s">
-        <v>1468</v>
+      <c r="G1480" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1480" s="8" t="s">
         <v>1473</v>
@@ -44018,8 +44021,8 @@
       <c r="F1483" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1483" s="4" t="s">
-        <v>1468</v>
+      <c r="G1483" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1483" s="8" t="s">
         <v>1473</v>
@@ -44044,8 +44047,8 @@
       <c r="F1484" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1484" s="4" t="s">
-        <v>1468</v>
+      <c r="G1484" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1484" s="8" t="s">
         <v>1473</v>
@@ -44148,8 +44151,8 @@
       <c r="F1488" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1488" s="4" t="s">
-        <v>1468</v>
+      <c r="G1488" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1488" s="8" t="s">
         <v>1473</v>
@@ -44538,8 +44541,8 @@
       <c r="F1503" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1503" s="4" t="s">
-        <v>1468</v>
+      <c r="G1503" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1503" s="8" t="s">
         <v>1473</v>
@@ -44665,8 +44668,8 @@
       <c r="F1508" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1508" s="4" t="s">
-        <v>1468</v>
+      <c r="G1508" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1508" s="8" t="s">
         <v>1473</v>
@@ -44948,8 +44951,8 @@
       <c r="F1519" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1519" s="4" t="s">
-        <v>1468</v>
+      <c r="G1519" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1519" s="8" t="s">
         <v>1473</v>
@@ -45208,8 +45211,8 @@
       <c r="F1529" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1529" s="4" t="s">
-        <v>1468</v>
+      <c r="G1529" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1529" s="8" t="s">
         <v>1473</v>
@@ -45260,8 +45263,8 @@
       <c r="F1531" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1531" s="4" t="s">
-        <v>1468</v>
+      <c r="G1531" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1531" s="8" t="s">
         <v>1473</v>
@@ -45462,8 +45465,8 @@
       <c r="F1539" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1539" s="4" t="s">
-        <v>1468</v>
+      <c r="G1539" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1539" s="8" t="s">
         <v>1473</v>
@@ -45540,8 +45543,8 @@
       <c r="F1542" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1542" s="4" t="s">
-        <v>1468</v>
+      <c r="G1542" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1542" s="8" t="s">
         <v>1473</v>
@@ -45693,8 +45696,8 @@
       <c r="F1548" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1548" s="4" t="s">
-        <v>1468</v>
+      <c r="G1548" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1548" s="8" t="s">
         <v>1473</v>
@@ -45719,8 +45722,8 @@
       <c r="F1549" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1549" s="4" t="s">
-        <v>1468</v>
+      <c r="G1549" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1549" s="8" t="s">
         <v>1473</v>
@@ -45771,8 +45774,8 @@
       <c r="F1551" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1551" s="4" t="s">
-        <v>1468</v>
+      <c r="G1551" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1551" s="8" t="s">
         <v>1473</v>
@@ -46135,8 +46138,8 @@
       <c r="F1565" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1565" s="4" t="s">
-        <v>1468</v>
+      <c r="G1565" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1565" s="8" t="s">
         <v>1473</v>
@@ -46161,8 +46164,8 @@
       <c r="F1566" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1566" s="4" t="s">
-        <v>1468</v>
+      <c r="G1566" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1566" s="8" t="s">
         <v>1473</v>
@@ -48079,8 +48082,8 @@
       <c r="F1640" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1640" s="4" t="s">
-        <v>1468</v>
+      <c r="G1640" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1640" s="8" t="s">
         <v>1473</v>
@@ -48414,8 +48417,8 @@
       <c r="F1653" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1653" s="4" t="s">
-        <v>1468</v>
+      <c r="G1653" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1653" s="4" t="s">
         <v>1473</v>
@@ -48492,8 +48495,8 @@
       <c r="F1656" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1656" s="4" t="s">
-        <v>1468</v>
+      <c r="G1656" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1656" s="4" t="s">
         <v>1473</v>
@@ -48518,8 +48521,8 @@
       <c r="F1657" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1657" s="4" t="s">
-        <v>1468</v>
+      <c r="G1657" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1657" s="4" t="s">
         <v>1473</v>
@@ -48570,8 +48573,8 @@
       <c r="F1659" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1659" s="4" t="s">
-        <v>1468</v>
+      <c r="G1659" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1659" s="4" t="s">
         <v>1473</v>
@@ -48596,8 +48599,8 @@
       <c r="F1660" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1660" s="4" t="s">
-        <v>1468</v>
+      <c r="G1660" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1660" s="4" t="s">
         <v>1473</v>
@@ -48622,8 +48625,8 @@
       <c r="F1661" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1661" s="4" t="s">
-        <v>1468</v>
+      <c r="G1661" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1661" s="4" t="s">
         <v>1473</v>
@@ -48934,8 +48937,8 @@
       <c r="F1673" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1673" s="4" t="s">
-        <v>1468</v>
+      <c r="G1673" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1673" s="4" t="s">
         <v>1473</v>
@@ -49116,8 +49119,8 @@
       <c r="F1680" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1680" s="4" t="s">
-        <v>1468</v>
+      <c r="G1680" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1680" s="4" t="s">
         <v>1473</v>
@@ -49194,8 +49197,8 @@
       <c r="F1683" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1683" s="4" t="s">
-        <v>1468</v>
+      <c r="G1683" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1683" s="4" t="s">
         <v>1473</v>
@@ -49272,8 +49275,8 @@
       <c r="F1686" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1686" s="4" t="s">
-        <v>1468</v>
+      <c r="G1686" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1686" s="4" t="s">
         <v>1473</v>
@@ -49376,8 +49379,8 @@
       <c r="F1690" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1690" s="4" t="s">
-        <v>1468</v>
+      <c r="G1690" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1690" s="4" t="s">
         <v>1473</v>
@@ -49558,8 +49561,8 @@
       <c r="F1697" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1697" s="4" t="s">
-        <v>1468</v>
+      <c r="G1697" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1697" s="4" t="s">
         <v>1473</v>
@@ -49584,8 +49587,8 @@
       <c r="F1698" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1698" s="4" t="s">
-        <v>1468</v>
+      <c r="G1698" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1698" s="4" t="s">
         <v>1473</v>
@@ -49610,8 +49613,8 @@
       <c r="F1699" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1699" s="4" t="s">
-        <v>1468</v>
+      <c r="G1699" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1699" s="4" t="s">
         <v>1473</v>
@@ -49792,8 +49795,8 @@
       <c r="F1706" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1706" s="4" t="s">
-        <v>1468</v>
+      <c r="G1706" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1706" s="4" t="s">
         <v>1473</v>
@@ -49818,8 +49821,8 @@
       <c r="F1707" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1707" s="4" t="s">
-        <v>1468</v>
+      <c r="G1707" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1707" s="4" t="s">
         <v>1473</v>
@@ -49844,8 +49847,8 @@
       <c r="F1708" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1708" s="4" t="s">
-        <v>1468</v>
+      <c r="G1708" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1708" s="4" t="s">
         <v>1473</v>
@@ -49870,8 +49873,8 @@
       <c r="F1709" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1709" s="4" t="s">
-        <v>1468</v>
+      <c r="G1709" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1709" s="4" t="s">
         <v>1473</v>
@@ -49896,8 +49899,8 @@
       <c r="F1710" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1710" s="4" t="s">
-        <v>1468</v>
+      <c r="G1710" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1710" s="4" t="s">
         <v>1473</v>
@@ -49922,8 +49925,8 @@
       <c r="F1711" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1711" s="4" t="s">
-        <v>1468</v>
+      <c r="G1711" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1711" s="4" t="s">
         <v>1473</v>
@@ -49948,8 +49951,8 @@
       <c r="F1712" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1712" s="4" t="s">
-        <v>1468</v>
+      <c r="G1712" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1712" s="4" t="s">
         <v>1473</v>
@@ -50000,8 +50003,8 @@
       <c r="F1714" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1714" s="4" t="s">
-        <v>1468</v>
+      <c r="G1714" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1714" s="4" t="s">
         <v>1473</v>
@@ -50052,8 +50055,8 @@
       <c r="F1716" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1716" s="4" t="s">
-        <v>1468</v>
+      <c r="G1716" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1716" s="4" t="s">
         <v>1473</v>
@@ -52132,8 +52135,8 @@
       <c r="F1796" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1796" s="4" t="s">
-        <v>1468</v>
+      <c r="G1796" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1796" s="4" t="s">
         <v>1473</v>
@@ -52444,8 +52447,8 @@
       <c r="F1808" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1808" s="4" t="s">
-        <v>1468</v>
+      <c r="G1808" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1808" s="4" t="s">
         <v>1473</v>
@@ -52704,8 +52707,8 @@
       <c r="F1818" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1818" s="4" t="s">
-        <v>1468</v>
+      <c r="G1818" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1818" s="4" t="s">
         <v>1473</v>
@@ -53094,8 +53097,8 @@
       <c r="F1833" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1833" s="4" t="s">
-        <v>1468</v>
+      <c r="G1833" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1833" s="4" t="s">
         <v>1473</v>
@@ -53146,8 +53149,8 @@
       <c r="F1835" s="5" t="s">
         <v>1467</v>
       </c>
-      <c r="G1835" s="4" t="s">
-        <v>1468</v>
+      <c r="G1835" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1835" s="5" t="s">
         <v>1473</v>
@@ -53172,8 +53175,8 @@
       <c r="F1836" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G1836" s="4" t="s">
-        <v>1468</v>
+      <c r="G1836" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1836" s="4" t="s">
         <v>1473</v>
@@ -53224,8 +53227,8 @@
       <c r="F1838" s="6" t="s">
         <v>1467</v>
       </c>
-      <c r="G1838" s="4" t="s">
-        <v>1468</v>
+      <c r="G1838" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1838" s="6" t="s">
         <v>1473</v>
@@ -53276,8 +53279,8 @@
       <c r="F1840" s="6" t="s">
         <v>1467</v>
       </c>
-      <c r="G1840" s="4" t="s">
-        <v>1468</v>
+      <c r="G1840" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1840" s="6" t="s">
         <v>1473</v>
@@ -53302,8 +53305,8 @@
       <c r="F1841" s="5" t="s">
         <v>1467</v>
       </c>
-      <c r="G1841" s="4" t="s">
-        <v>1468</v>
+      <c r="G1841" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1841" s="5" t="s">
         <v>1473</v>
@@ -54706,8 +54709,8 @@
       <c r="F1895" s="5" t="s">
         <v>1467</v>
       </c>
-      <c r="G1895" s="4" t="s">
-        <v>1468</v>
+      <c r="G1895" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1895" s="5" t="s">
         <v>1473</v>
@@ -55148,8 +55151,8 @@
       <c r="F1912" s="6" t="s">
         <v>1467</v>
       </c>
-      <c r="G1912" s="4" t="s">
-        <v>1468</v>
+      <c r="G1912" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K1912" s="6" t="s">
         <v>1473</v>
@@ -57904,8 +57907,8 @@
       <c r="F2018" s="6" t="s">
         <v>1467</v>
       </c>
-      <c r="G2018" s="4" t="s">
-        <v>1468</v>
+      <c r="G2018" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2018" s="6" t="s">
         <v>1473</v>
@@ -57930,8 +57933,8 @@
       <c r="F2019" s="5" t="s">
         <v>1467</v>
       </c>
-      <c r="G2019" s="4" t="s">
-        <v>1468</v>
+      <c r="G2019" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2019" s="5" t="s">
         <v>1473</v>
@@ -58996,8 +58999,8 @@
       <c r="F2060" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2060" s="4" t="s">
-        <v>1468</v>
+      <c r="G2060" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2060" s="4" t="s">
         <v>1473</v>
@@ -59178,8 +59181,8 @@
       <c r="F2067" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2067" s="4" t="s">
-        <v>1468</v>
+      <c r="G2067" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2067" s="4" t="s">
         <v>1473</v>
@@ -59282,8 +59285,8 @@
       <c r="F2071" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2071" s="4" t="s">
-        <v>1468</v>
+      <c r="G2071" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2071" s="4" t="s">
         <v>1473</v>
@@ -59490,8 +59493,8 @@
       <c r="F2079" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2079" s="4" t="s">
-        <v>1468</v>
+      <c r="G2079" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2079" s="4" t="s">
         <v>1473</v>
@@ -59776,8 +59779,8 @@
       <c r="F2090" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2090" s="4" t="s">
-        <v>1468</v>
+      <c r="G2090" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2090" s="4" t="s">
         <v>1473</v>
@@ -60010,8 +60013,8 @@
       <c r="F2099" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2099" s="4" t="s">
-        <v>1468</v>
+      <c r="G2099" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2099" s="4" t="s">
         <v>1473</v>
@@ -60036,8 +60039,8 @@
       <c r="F2100" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2100" s="4" t="s">
-        <v>1468</v>
+      <c r="G2100" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2100" s="4" t="s">
         <v>1473</v>
@@ -60088,8 +60091,8 @@
       <c r="F2102" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2102" s="4" t="s">
-        <v>1468</v>
+      <c r="G2102" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2102" s="4" t="s">
         <v>1473</v>
@@ -60192,8 +60195,8 @@
       <c r="F2106" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2106" s="4" t="s">
-        <v>1468</v>
+      <c r="G2106" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2106" s="4" t="s">
         <v>1473</v>
@@ -60218,8 +60221,8 @@
       <c r="F2107" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2107" s="4" t="s">
-        <v>1468</v>
+      <c r="G2107" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2107" s="4" t="s">
         <v>1473</v>
@@ -60244,8 +60247,8 @@
       <c r="F2108" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2108" s="4" t="s">
-        <v>1468</v>
+      <c r="G2108" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2108" s="8" t="s">
         <v>1473</v>
@@ -60634,8 +60637,8 @@
       <c r="F2123" s="4" t="s">
         <v>1467</v>
       </c>
-      <c r="G2123" s="4" t="s">
-        <v>1468</v>
+      <c r="G2123" s="10" t="s">
+        <v>1477</v>
       </c>
       <c r="K2123" s="4" t="s">
         <v>1473</v>

</xml_diff>

<commit_message>
feat: complete UI logic for pagu historis chart and PDF, format numbers, fix AI fallback and PDF auto page break
</commit_message>
<xml_diff>
--- a/db.xlsx
+++ b/db.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BK\OneDrive - UGM 365\Desktop\verifikasi-online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A80717-36DE-4AAC-AA0C-A1BB2EE6EACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A3CF508-822E-46E4-83BA-8B3343EF9222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{14108520-BF54-4EAA-92D2-D404123A5DCA}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">pagu!$A$1:$K$2132</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4567,7 +4568,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>